<commit_message>
Updated PHL_grids_kan model - 2026-05-06 23:19
</commit_message>
<xml_diff>
--- a/VerveStacks_PHL_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_PHL_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_PHL_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1BCB884D-243E-41CC-8F33-A498C74C0614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE74DDAC-9451-449A-A63D-9868667F1582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5398,7 +5398,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D86E9EFF-FD0C-47D3-90FF-24406B4DFF82}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5613C46-131E-4350-8114-8ADA1FBD325B}">
   <dimension ref="B9:H366"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -32356,7 +32356,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA5AB38F-4A2F-428F-8893-6D0B6289C8BD}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC862623-7AEE-44D0-9725-51FEF4044487}">
   <dimension ref="B9:L366"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>